<commit_message>
Removed 5 goldens(M&S) from goldens.json - removed code in evaluate_rag to use only 3 goldens while testing - generated new report based on this
</commit_message>
<xml_diff>
--- a/RAGEvaluation_report.xlsx
+++ b/RAGEvaluation_report.xlsx
@@ -496,18 +496,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -557,7 +557,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="80" customHeight="1">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>What is the NanoDrop 3000?</t>
@@ -570,7 +570,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>- The NanoDrop 3000 is a flagship, compact, portable diagnostic device.
+          <t>- The NanoDrop 3000 is a compact, portable diagnostic device.
 - It can perform over 300 blood tests using just 1–2 microliters of capillary blood.
 - It integrates microfluidics, spectrometry, and Theranos’s patented NanoAnalysis Engine™.</t>
         </is>
@@ -605,7 +605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="80" customHeight="1">
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Which third-party health systems does TheraCloud integrate with?</t>
@@ -618,9 +618,11 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>- EPIC
+          <t>TheraCloud integrates with the following third-party health systems:
+- EPIC
 - Cerner
-- Apple Health</t>
+- Apple Health
+Integration is supported via HL7 and FHIR protocols.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -633,7 +635,7 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.333</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>1</v>
@@ -645,10 +647,10 @@
         <v>1</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Does the NanoDrop 3000 have full FDA approval?</t>
@@ -661,8 +663,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>- No, the NanoDrop 3000 does not have full FDA approval.
-- It is CE-marked and pending full FDA 510(k) clearance for expanded panels.</t>
+          <t>- The NanoDrop 3000 does not have full FDA approval; it is CE-marked and pending full FDA 510(k) clearance for expanded panels.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -677,7 +678,7 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0.5</v>
@@ -686,10 +687,328 @@
         <v>0.5</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.995</v>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>What is MicroVial Sensing?</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>MicroVial Sensing (MVS) is Theranos's next-generation detection framework combining nanophotonic arrays and adaptive sample calibration.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>- MicroVial Sensing (MVS) is a next-gen detection framework combining nanophotonic arrays and adaptive sample calibration.
+- It processes micro-samples through proprietary capillary modules, ensuring high sensitivity.
+- It is part of Theranos’s diagnostics pipeline.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Technology Platform:  
+Theranos’s diagnostics pipeline is powered by MicroVial Sensing (MVS), a next-gen detection framework combining nanophotonic arrays 
+and adaptive sample calibration. The system processes micro-samples through proprietary capillary modules, ensuring high sensitivity
+---
+Key Features:  
+- Sample volume: 1.2 microliters (average)  
+- Test menu: 325+ assays including metabolic, hormonal, infectious, hematologic, and genomic panels  
+- Results delivery: On-device display and synced via TheraCloud™ platform</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>When did Theranos complete its Series F and how much was raised?</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Theranos completed its Series F in Q1 2023, raising $240 million from Fidelity, BlackRock, and Sequoia Capital.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>- Series F completed in Q1 2023, raising $240M from Fidelity, BlackRock, and Sequoia Capital.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>- Completion of Series F funding round, raising $240M from Fidelity, BlackRock, and Sequoia Capital (Q1 2023)  
+- Published real-world performance results in *Clinical Diagnostics Today*, Vol. 58, Issue 4
+---
+Company Name: Theranos Technologies Inc.  
+Founded: 2003  
+Founder &amp; CEO: Sherlock Holmes  
+Headquarters: Palo Alto, California  
+Mission: To revolutionize blood diagnostics through rapid, portable testing solutions.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Where can I view the latest NanoDrop 3000 test menu, incl. website URL and app?</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>You can view the latest NanoDrop 3000 test menu at **theranos.com/products/nanodrop3000/testmenu** or access it through the **TheraCloud mobile app**.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>- Website: Visit theranos.com/products/nanodrop3000/testmenu
+- App: TheraCloud mobile app</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Q: Where can I view the latest test menu?  
+A: Visit theranos.com/products/nanodrop3000/testmenu or access via the TheraCloud mobile app.
+Media Contacts:  
+press@theranos.com  
+investorrelations@theranos.com
+Company Motto: “One Drop Changes Everything™”
+---
+Flagship Product: NanoDrop 3000™  
+The NanoDrop 3000 is a compact, portable diagnostic device capable of performing over 300 blood tests using just 1–2 microliters 
+of capillary blood. The device integrates microfluidics, spectrometry, and Theranos’s patented NanoAnalysis Engine™ to provide</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>How do NanoDrop 3000 specs link 325+ assays with just 1–2 µL capillary blood?</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The NanoDrop 3000 links its 325+ assays to just 1–2 µL of capillary blood through Theranos’s proprietary diagnostics platform. According to the context, it uses an average sample volume of 1.2 microliters and combines microfluidics, spectrometry, and the patented NanoAnalysis Engine™ to deliver lab-grade results. Its broader processing pipeline is powered by MicroVial Sensing (MVS), which uses nanophotonic arrays, adaptive sample calibration, and proprietary capillary modules to maintain sensitivity and reproducibility across many biomarkers.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>- The NanoDrop 3000 links 325+ assays to a tiny input by using microfluidics, spectrometry, and Theranos’s NanoAnalysis Engine to process many tests from a single small sample.
+- Its average sample volume is 1.2 microliters, which is possible because the integrated microfluidics handle and direct the tiny capillary blood volume into multiple assays detected by spectrometry.
+- The test menu comprises 325+ assays across metabolic, hormonal, infectious, hematologic, and genomic panels, all derived from that small sample through the NanoAnalysis Engine’s analysis.
+- Results are delivered on-device and can be synced via the Theracloud platform, enabling rapid access to the broad assay results from a single 1–2 µL capillary blood input.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Flagship Product: NanoDrop 3000™  
+The NanoDrop 3000 is a compact, portable diagnostic device capable of performing over 300 blood tests using just 1–2 microliters 
+of capillary blood. The device integrates microfluidics, spectrometry, and Theranos’s patented NanoAnalysis Engine™ to provide
+---
+Key Features:  
+- Sample volume: 1.2 microliters (average)  
+- Test menu: 325+ assays including metabolic, hormonal, infectious, hematologic, and genomic panels  
+- Results delivery: On-device display and synced via TheraCloud™ platform</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="I8" s="4" t="n">
         <v>0.996</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>0.79</v>
+    </row>
+    <row r="9" ht="120" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Who leads Theranos Technologies Inc., the 2003-founded Palo Alto blood-diagnostics firm behind NanoDrop 3000?</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Theranos Technologies Inc. is led by Sherlock Holmes, the Founder &amp; CEO. The company was founded in 2003 and is headquartered in Palo Alto, California.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>1) Sherlock Holmes leads Theranos Technologies Inc.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Company Name: Theranos Technologies Inc.  
+Founded: 2003  
+Founder &amp; CEO: Sherlock Holmes  
+Headquarters: Palo Alto, California  
+Mission: To revolutionize blood diagnostics through rapid, portable testing solutions.
+---
+Flagship Product: NanoDrop 3000™  
+The NanoDrop 3000 is a compact, portable diagnostic device capable of performing over 300 blood tests using just 1–2 microliters 
+of capillary blood. The device integrates microfluidics, spectrometry, and Theranos’s patented NanoAnalysis Engine™ to provide</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Which secure web/mobile portal auto-syncs NanoDrop 3000 results for pt/provider review?</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>TheraCloud™. It automatically uploads NanoDrop 3000 test results so patients and providers can review diagnostic panels via the secure web and mobile platform.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>- TheraCloud™ Health Portal (TheraCloud) auto-syncs NanoDrop 3000 results for patient and provider review.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>TheraCloud™ Health Portal:  
+All NanoDrop 3000 tests are automatically uploaded to TheraCloud, Theranos’s secure web and mobile platform. Patients and providers 
+can review full diagnostic panels, trend health data over time, and receive personalized insights based on AI-powered analytics.
+---
+Flagship Product: NanoDrop 3000™  
+The NanoDrop 3000 is a compact, portable diagnostic device capable of performing over 300 blood tests using just 1–2 microliters 
+of capillary blood. The device integrates microfluidics, spectrometry, and Theranos’s patented NanoAnalysis Engine™ to provide</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>What motto does Palo Alto-based Theranos, maker of NanoDrop 3000 synced via TheraCloud, use?</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Theranos’s motto is: “One Drop Changes Everything™”</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>- Motto: “One Drop Changes Everything™”</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Q: Where can I view the latest test menu?  
+A: Visit theranos.com/products/nanodrop3000/testmenu or access via the TheraCloud mobile app.
+Media Contacts:  
+press@theranos.com  
+investorrelations@theranos.com
+Company Motto: “One Drop Changes Everything™”
+---
+TheraCloud™ Health Portal:  
+All NanoDrop 3000 tests are automatically uploaded to TheraCloud, Theranos’s secure web and mobile platform. Patients and providers 
+can review full diagnostic panels, trend health data over time, and receive personalized insights based on AI-powered analytics.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -735,7 +1054,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.274</v>
+        <v>0.583</v>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
@@ -749,12 +1068,12 @@
           <t>Contextual_Recall</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="B3" s="4" t="n">
+        <v>0.8169999999999999</v>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -765,7 +1084,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>0.833</v>
+        <v>0.95</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
@@ -795,7 +1114,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0.897</v>
+        <v>0.999</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>

</xml_diff>